<commit_message>
Improve notebook with NumPy docstrings, error handling, and retry logic
- Add NumPy-style docstring to get_pc_data with Parameters, Returns, Raises
- Add retry logic with backoff for PubChem 503/429 rate-limit errors
- Add per-item progress printing in all API loops
- Add CID fallback: use name CID when CAS CID resolves to 0
- Fix pc_cas initialized as list instead of string
- Remove unused imports (sys, re, math, numpy)
- Remove unused iupac variable
- Wrap all key access in try/except for missing PubChem sections
- Sort GHS hazards and CAS numbers for stable output
- Add .gitignore; untrack __pycache__ files
- Regenerate output files with improved logic

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PubChem_output1.xlsx
+++ b/PubChem_output1.xlsx
@@ -492,37 +492,57 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Nonaethylene Glycol Nonylphenyl Ether</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>26571-11-9</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>14409-72-4
+26027-38-3</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>None</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Nonoxynol-9
+ToDay
+Delfen
+26571-11-9
+Nonaethylene glycol nonylphenyl ether</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Corrosive
+Environmental Hazard
+Irritant</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>H302 (100%): Harmful if swallowed [Warning Acute toxicity, oral]
+H302 (80.3%): Harmful if swallowed [Warning Acute toxicity, oral]
+H302: Harmful if swallowed [Warning Acute toxicity, oral]
+H315 (100%): Causes skin irritation [Warning Skin corrosion/irritation]
+H315 (75.4%): Causes skin irritation [Warning Skin corrosion/irritation]
+H315: Causes skin irritation [Warning Skin corrosion/irritation]
+H318 (80.3%): Causes serious eye damage [Danger Serious eye damage/eye irritation]
+H318: Causes serious eye damage [Danger Serious eye damage/eye irritation]
+H319 (100%): Causes serious eye irritation [Warning Serious eye damage/eye irritation]
+H319 (19.7%): Causes serious eye irritation [Warning Serious eye damage/eye irritation]
+H319: Causes serious eye irritation [Warning Serious eye damage/eye irritation]
+H411 (100%): Toxic to aquatic life with long lasting effects [Hazardous to the aquatic environment, long-term hazard]
+H411 (48.8%): Toxic to aquatic life with long lasting effects [Hazardous to the aquatic environment, long-term hazard]
+H412 (31.5%): Harmful to aquatic life with long lasting effects [Hazardous to the aquatic environment, long-term hazard]</t>
         </is>
       </c>
     </row>
@@ -555,7 +575,8 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>9082-06-8</t>
+          <t>9082-06-8
+91079-40-2</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -581,34 +602,34 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>H315: Causes skin irritation [Warning Skin corrosion/irritation]
-H370: Causes damage to organs [Danger Specific target organ toxicity, single exposure]
-H350: May cause cancer [Danger Carcinogenicity]
-H301 (94.8%): Toxic if swallowed [Danger Acute toxicity, oral]
+          <t>H301 (94.8%): Toxic if swallowed [Danger Acute toxicity, oral]
+H301: Toxic if swallowed [Danger Acute toxicity, oral]
+H311: Toxic in contact with skin [Danger Acute toxicity, dermal]
+H312 (94.2%): Harmful in contact with skin [Warning Acute toxicity, dermal]
+H312: Harmful in contact with skin [Warning Acute toxicity, dermal]
 H315 (96.2%): Causes skin irritation [Warning Skin corrosion/irritation]
-H361 (94.1%): Suspected of damaging fertility or the unborn child [Warning Reproductive toxicity]
+H315: Causes skin irritation [Warning Skin corrosion/irritation]
+H316: Causes mild skin irritation [Warning Skin corrosion/irritation]
 H317 (96.2%): May cause an allergic skin reaction [Warning Sensitization, Skin]
+H317: May cause an allergic skin reaction [Warning Sensitization, Skin]
+H319 (96%): Causes serious eye irritation [Warning Serious eye damage/eye irritation]
+H319: Causes serious eye irritation [Warning Serious eye damage/eye irritation]
+H332 (94.6%): Harmful if inhaled [Warning Acute toxicity, inhalation]
 H332: Harmful if inhaled [Warning Acute toxicity, inhalation]
-H319 (96%): Causes serious eye irritation [Warning Serious eye damage/eye irritation]
 H340 (96.2%): May cause genetic defects [Danger Germ cell mutagenicity]
-H319: Causes serious eye irritation [Warning Serious eye damage/eye irritation]
-H372 **: Causes damage to organs through prolonged or repeated exposure [Danger Specific target organ toxicity, repeated exposure]
 H340: May cause genetic defects [Danger Germ cell mutagenicity]
 H350 (96.1%): May cause cancer [Danger Carcinogenicity]
-H402: Harmful to aquatic life [Hazardous to the aquatic environment, acute hazard]
-H311: Toxic in contact with skin [Danger Acute toxicity, dermal]
-H332 (94.6%): Harmful if inhaled [Warning Acute toxicity, inhalation]
-H301: Toxic if swallowed [Danger Acute toxicity, oral]
+H350: May cause cancer [Danger Carcinogenicity]
+H360: May damage fertility or the unborn child [Danger Reproductive toxicity]
+H361 (94.1%): Suspected of damaging fertility or the unborn child [Warning Reproductive toxicity]
+H361: Suspected of damaging fertility or the unborn child [Warning Reproductive toxicity]
+H361f ***: Suspected of damaging fertility [Warning Reproductive toxicity]
+H361f: Suspected of damaging fertility [Warning Reproductive toxicity]
+H370: Causes damage to organs [Danger Specific target organ toxicity, single exposure]
 H372 (94.8%): Causes damage to organs through prolonged or repeated exposure [Danger Specific target organ toxicity, repeated exposure]
-H312: Harmful in contact with skin [Warning Acute toxicity, dermal]
-H361: Suspected of damaging fertility or the unborn child [Warning Reproductive toxicity]
+H372 **: Causes damage to organs through prolonged or repeated exposure [Danger Specific target organ toxicity, repeated exposure]
 H372: Causes damage to organs through prolonged or repeated exposure [Danger Specific target organ toxicity, repeated exposure]
-H360: May damage fertility or the unborn child [Danger Reproductive toxicity]
-H312 (94.2%): Harmful in contact with skin [Warning Acute toxicity, dermal]
-H316: Causes mild skin irritation [Warning Skin corrosion/irritation]
-H361f: Suspected of damaging fertility [Warning Reproductive toxicity]
-H361f ***: Suspected of damaging fertility [Warning Reproductive toxicity]
-H317: May cause an allergic skin reaction [Warning Sensitization, Skin]</t>
+H402: Harmful to aquatic life [Hazardous to the aquatic environment, acute hazard]</t>
         </is>
       </c>
     </row>
@@ -641,10 +662,10 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>39377-45-2
+          <t>12174-49-1
 12522-88-2
-90669-62-8
-12174-49-1</t>
+39377-45-2
+90669-62-8</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -655,8 +676,8 @@
       <c r="I4" t="inlineStr">
         <is>
           <t>ALUMINUM OXIDE
+1344-28-1
 Aluminium oxide
-1344-28-1
 Aloxite
 gamma-Alumina</t>
         </is>
@@ -670,9 +691,9 @@
       <c r="K4" t="inlineStr">
         <is>
           <t>H335 (100%): May cause respiratory irritation [Warning Specific target organ toxicity, single exposure; Respiratory tract irritation]
-H373 (100%): May causes damage to organs through prolonged or repeated exposure [Warning Specific target organ toxicity, repeated exposure]
 H335: May cause respiratory irritation [Warning Specific target organ toxicity, single exposure; Respiratory tract irritation]
-H372: Causes damage to organs through prolonged or repeated exposure [Danger Specific target organ toxicity, repeated exposure]</t>
+H372: Causes damage to organs through prolonged or repeated exposure [Danger Specific target organ toxicity, repeated exposure]
+H373 (100%): May causes damage to organs through prolonged or repeated exposure [Warning Specific target organ toxicity, repeated exposure]</t>
         </is>
       </c>
     </row>
@@ -725,39 +746,39 @@
       <c r="J5" t="inlineStr">
         <is>
           <t>Acute Toxic
+Corrosive
 Health Hazard
-Irritant
-Corrosive</t>
+Irritant</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>H315: Causes skin irritation [Warning Skin corrosion/irritation]
-H370: Causes damage to organs [Danger Specific target organ toxicity, single exposure]
-H331 (11.7%): Toxic if inhaled [Danger Acute toxicity, inhalation]
-H330: Fatal if inhaled [Danger Acute toxicity, inhalation]
+          <t>H227: Combustible liquid [Warning Flammable liquids]
+H302 (12.4%): Harmful if swallowed [Warning Acute toxicity, oral]
+H302 (99.5%): Harmful if swallowed [Warning Acute toxicity, oral]
+H302: Harmful if swallowed [Warning Acute toxicity, oral]
+H310: Fatal in contact with skin [Danger Acute toxicity, dermal]
+H311: Toxic in contact with skin [Danger Acute toxicity, dermal]
+H312 (11.1%): Harmful in contact with skin [Warning Acute toxicity, dermal]
+H312 (79.9%): Harmful in contact with skin [Warning Acute toxicity, dermal]
+H312: Harmful in contact with skin [Warning Acute toxicity, dermal]
+H315 (99.6%): Causes skin irritation [Warning Skin corrosion/irritation]
+H315: Causes skin irritation [Warning Skin corrosion/irritation]
+H318 (38.9%): Causes serious eye damage [Danger Serious eye damage/eye irritation]
 H319 (37.3%): Causes serious eye irritation [Warning Serious eye damage/eye irritation]
-H302: Harmful if swallowed [Warning Acute toxicity, oral]
-H335: May cause respiratory irritation [Warning Specific target organ toxicity, single exposure; Respiratory tract irritation]
-H315 (99.6%): Causes skin irritation [Warning Skin corrosion/irritation]
-H332: Harmful if inhaled [Warning Acute toxicity, inhalation]
-H312 (11.1%): Harmful in contact with skin [Warning Acute toxicity, dermal]
-H373: May causes damage to organs through prolonged or repeated exposure [Warning Specific target organ toxicity, repeated exposure]
-H336: May cause drowsiness or dizziness [Warning Specific target organ toxicity, single exposure; Narcotic effects]
 H319 (99.5%): Causes serious eye irritation [Warning Serious eye damage/eye irritation]
 H319: Causes serious eye irritation [Warning Serious eye damage/eye irritation]
-H302 (12.4%): Harmful if swallowed [Warning Acute toxicity, oral]
-H302 (99.5%): Harmful if swallowed [Warning Acute toxicity, oral]
-H227: Combustible liquid [Warning Flammable liquids]
+H330: Fatal if inhaled [Danger Acute toxicity, inhalation]
+H331 (11.7%): Toxic if inhaled [Danger Acute toxicity, inhalation]
 H331: Toxic if inhaled [Danger Acute toxicity, inhalation]
-H311: Toxic in contact with skin [Danger Acute toxicity, dermal]
-H312 (79.9%): Harmful in contact with skin [Warning Acute toxicity, dermal]
-H312: Harmful in contact with skin [Warning Acute toxicity, dermal]
+H332 (83.6%): Harmful if inhaled [Warning Acute toxicity, inhalation]
+H332: Harmful if inhaled [Warning Acute toxicity, inhalation]
+H335: May cause respiratory irritation [Warning Specific target organ toxicity, single exposure; Respiratory tract irritation]
+H336: May cause drowsiness or dizziness [Warning Specific target organ toxicity, single exposure; Narcotic effects]
 H361: Suspected of damaging fertility or the unborn child [Warning Reproductive toxicity]
-H318 (38.9%): Causes serious eye damage [Danger Serious eye damage/eye irritation]
+H370: Causes damage to organs [Danger Specific target organ toxicity, single exposure]
 H372: Causes damage to organs through prolonged or repeated exposure [Danger Specific target organ toxicity, repeated exposure]
-H332 (83.6%): Harmful if inhaled [Warning Acute toxicity, inhalation]
-H310: Fatal in contact with skin [Danger Acute toxicity, dermal]</t>
+H373: May causes damage to organs through prolonged or repeated exposure [Warning Specific target organ toxicity, repeated exposure]</t>
         </is>
       </c>
     </row>
@@ -790,8 +811,8 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>88357-62-4
-822-06-0, 11142-52-2</t>
+          <t>822-06-0, 11142-52-2
+88357-62-4</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -811,34 +832,34 @@
       <c r="J6" t="inlineStr">
         <is>
           <t>Acute Toxic
+Corrosive
 Health Hazard
-Irritant
-Corrosive</t>
+Irritant</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>H315: Causes skin irritation [Warning Skin corrosion/irritation]
+          <t>H302 (78.6%): Harmful if swallowed [Warning Acute toxicity, oral]
+H302: Harmful if swallowed [Warning Acute toxicity, oral]
+H311: Toxic in contact with skin [Danger Acute toxicity, dermal]
+H314: Causes severe skin burns and eye damage [Danger Skin corrosion/irritation]
+H315 (97.2%): Causes skin irritation [Warning Skin corrosion/irritation]
+H315: Causes skin irritation [Warning Skin corrosion/irritation]
+H317 (&gt; 99.9%): May cause an allergic skin reaction [Warning Sensitization, Skin]
+H317: May cause an allergic skin reaction [Warning Sensitization, Skin]
+H318: Causes serious eye damage [Danger Serious eye damage/eye irritation]
 H319 (97.3%): Causes serious eye irritation [Warning Serious eye damage/eye irritation]
+H319: Causes serious eye irritation [Warning Serious eye damage/eye irritation]
+H330 (77%): Fatal if inhaled [Danger Acute toxicity, inhalation]
+H330: Fatal if inhaled [Danger Acute toxicity, inhalation]
+H331 (23.5%): Toxic if inhaled [Danger Acute toxicity, inhalation]
+H331: Toxic if inhaled [Danger Acute toxicity, inhalation]
+H334 (&gt; 99.9%): May cause allergy or asthma symptoms or breathing difficulties if inhaled [Danger Sensitization, respiratory]
+H334: May cause allergy or asthma symptoms or breathing difficulties if inhaled [Danger Sensitization, respiratory]
 H335 (97.5%): May cause respiratory irritation [Warning Specific target organ toxicity, single exposure; Respiratory tract irritation]
+H335: May cause respiratory irritation [Warning Specific target organ toxicity, single exposure; Respiratory tract irritation]
 H370: Causes damage to organs [Danger Specific target organ toxicity, single exposure]
-H334: May cause allergy or asthma symptoms or breathing difficulties if inhaled [Danger Sensitization, respiratory]
-H330: Fatal if inhaled [Danger Acute toxicity, inhalation]
-H302: Harmful if swallowed [Warning Acute toxicity, oral]
-H335: May cause respiratory irritation [Warning Specific target organ toxicity, single exposure; Respiratory tract irritation]
-H331 (23.5%): Toxic if inhaled [Danger Acute toxicity, inhalation]
-H318: Causes serious eye damage [Danger Serious eye damage/eye irritation]
-H319: Causes serious eye irritation [Warning Serious eye damage/eye irritation]
-H334 (&gt; 99.9%): May cause allergy or asthma symptoms or breathing difficulties if inhaled [Danger Sensitization, respiratory]
-H314: Causes severe skin burns and eye damage [Danger Skin corrosion/irritation]
-H331: Toxic if inhaled [Danger Acute toxicity, inhalation]
-H311: Toxic in contact with skin [Danger Acute toxicity, dermal]
-H330 (77%): Fatal if inhaled [Danger Acute toxicity, inhalation]
-H302 (78.6%): Harmful if swallowed [Warning Acute toxicity, oral]
-H372: Causes damage to organs through prolonged or repeated exposure [Danger Specific target organ toxicity, repeated exposure]
-H317 (&gt; 99.9%): May cause an allergic skin reaction [Warning Sensitization, Skin]
-H315 (97.2%): Causes skin irritation [Warning Skin corrosion/irritation]
-H317: May cause an allergic skin reaction [Warning Sensitization, Skin]</t>
+H372: Causes damage to organs through prolonged or repeated exposure [Danger Specific target organ toxicity, repeated exposure]</t>
         </is>
       </c>
     </row>
@@ -864,36 +885,12 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -913,36 +910,12 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>